<commit_message>
Modelos constreñidos con glucosa y biomasa
</commit_message>
<xml_diff>
--- a/Data/HPLC_results/Resultados_Procesados.xlsx
+++ b/Data/HPLC_results/Resultados_Procesados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\yannis\CNB\CNB\Data\HPLC_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E7CA68-D27F-4FF9-8CB4-E0854E7CDD2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25B53B9C-12AC-4023-ADD7-9E6EF2BD9694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="10032" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -154,12 +154,42 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -189,11 +219,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,929 +532,1663 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:AV22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="14" max="14" width="8.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7"/>
+      <c r="Z1" s="7"/>
+      <c r="AA1" s="7"/>
+      <c r="AB1" s="7"/>
+      <c r="AC1" s="7"/>
+      <c r="AD1" s="7"/>
+      <c r="AE1" s="7"/>
+      <c r="AF1" s="7"/>
+      <c r="AG1" s="7"/>
+      <c r="AH1" s="7"/>
+      <c r="AI1" s="7"/>
+      <c r="AJ1" s="7"/>
+      <c r="AK1" s="7"/>
+      <c r="AL1" s="7"/>
+      <c r="AM1" s="7"/>
+      <c r="AN1" s="7"/>
+      <c r="AO1" s="7"/>
+      <c r="AP1" s="7"/>
+      <c r="AQ1" s="7"/>
+      <c r="AR1" s="7"/>
+      <c r="AS1" s="7"/>
+      <c r="AT1" s="7"/>
+      <c r="AU1" s="7"/>
+      <c r="AV1" s="7"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2">
+    <row r="2" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
+      <c r="D2" s="6">
+        <v>0</v>
+      </c>
+      <c r="E2" s="6">
         <v>0.02</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="6">
         <v>31.310951541023801</v>
       </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
+      <c r="G2" s="6">
+        <v>0</v>
+      </c>
+      <c r="H2" s="6">
+        <v>0</v>
+      </c>
+      <c r="I2" s="6">
+        <v>0</v>
+      </c>
+      <c r="J2" s="6">
+        <v>0</v>
+      </c>
+      <c r="K2" s="6">
+        <v>0</v>
+      </c>
+      <c r="L2" s="6">
+        <v>0</v>
+      </c>
+      <c r="M2" s="6">
+        <v>0</v>
+      </c>
+      <c r="N2" s="6"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
+      <c r="U2" s="7"/>
+      <c r="V2" s="7"/>
+      <c r="W2" s="7"/>
+      <c r="X2" s="7"/>
+      <c r="Y2" s="7"/>
+      <c r="Z2" s="7"/>
+      <c r="AA2" s="7"/>
+      <c r="AB2" s="7"/>
+      <c r="AC2" s="7"/>
+      <c r="AD2" s="7"/>
+      <c r="AE2" s="7"/>
+      <c r="AF2" s="7"/>
+      <c r="AG2" s="7"/>
+      <c r="AH2" s="7"/>
+      <c r="AI2" s="7"/>
+      <c r="AJ2" s="7"/>
+      <c r="AK2" s="7"/>
+      <c r="AL2" s="7"/>
+      <c r="AM2" s="7"/>
+      <c r="AN2" s="7"/>
+      <c r="AO2" s="7"/>
+      <c r="AP2" s="7"/>
+      <c r="AQ2" s="7"/>
+      <c r="AR2" s="7"/>
+      <c r="AS2" s="7"/>
+      <c r="AT2" s="7"/>
+      <c r="AU2" s="7"/>
+      <c r="AV2" s="7"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="3" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>5.33</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>0.151</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="1">
         <v>23.858350949006802</v>
       </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
         <v>0.15667318344737699</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="1">
         <v>-22.111470224480449</v>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0</v>
+      </c>
+      <c r="M3" s="1">
         <v>0.46484101596455668</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="1">
         <v>3.323128875503923E-2</v>
       </c>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="7"/>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="7"/>
+      <c r="AB3" s="7"/>
+      <c r="AC3" s="7"/>
+      <c r="AD3" s="7"/>
+      <c r="AE3" s="7"/>
+      <c r="AF3" s="7"/>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="7"/>
+      <c r="AI3" s="7"/>
+      <c r="AJ3" s="7"/>
+      <c r="AK3" s="7"/>
+      <c r="AL3" s="7"/>
+      <c r="AM3" s="7"/>
+      <c r="AN3" s="7"/>
+      <c r="AO3" s="7"/>
+      <c r="AP3" s="7"/>
+      <c r="AQ3" s="7"/>
+      <c r="AR3" s="7"/>
+      <c r="AS3" s="7"/>
+      <c r="AT3" s="7"/>
+      <c r="AU3" s="7"/>
+      <c r="AV3" s="7"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="4" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>6.58</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>0.36499999999999999</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="1">
         <v>22.202016683774101</v>
       </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
         <v>0.32936787227109798</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="1">
         <v>-6.9441863199999192</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1">
         <v>0.72402299513971924</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="1">
         <v>0.2314764737696052</v>
       </c>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="7"/>
+      <c r="V4" s="7"/>
+      <c r="W4" s="7"/>
+      <c r="X4" s="7"/>
+      <c r="Y4" s="7"/>
+      <c r="Z4" s="7"/>
+      <c r="AA4" s="7"/>
+      <c r="AB4" s="7"/>
+      <c r="AC4" s="7"/>
+      <c r="AD4" s="7"/>
+      <c r="AE4" s="7"/>
+      <c r="AF4" s="7"/>
+      <c r="AG4" s="7"/>
+      <c r="AH4" s="7"/>
+      <c r="AI4" s="7"/>
+      <c r="AJ4" s="7"/>
+      <c r="AK4" s="7"/>
+      <c r="AL4" s="7"/>
+      <c r="AM4" s="7"/>
+      <c r="AN4" s="7"/>
+      <c r="AO4" s="7"/>
+      <c r="AP4" s="7"/>
+      <c r="AQ4" s="7"/>
+      <c r="AR4" s="7"/>
+      <c r="AS4" s="7"/>
+      <c r="AT4" s="7"/>
+      <c r="AU4" s="7"/>
+      <c r="AV4" s="7"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5">
+    <row r="5" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="1">
         <v>7.33</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>0.59199999999999997</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="1">
         <v>20.9177049666316</v>
       </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1">
         <v>-4.8387182736994934</v>
       </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
+      <c r="K5" s="1">
+        <v>0</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0</v>
+      </c>
+      <c r="M5" s="1">
         <v>-1.2409124054973111</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="1">
         <v>0.40923021453037672</v>
       </c>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="7"/>
+      <c r="T5" s="7"/>
+      <c r="U5" s="7"/>
+      <c r="V5" s="7"/>
+      <c r="W5" s="7"/>
+      <c r="X5" s="7"/>
+      <c r="Y5" s="7"/>
+      <c r="Z5" s="7"/>
+      <c r="AA5" s="7"/>
+      <c r="AB5" s="7"/>
+      <c r="AC5" s="7"/>
+      <c r="AD5" s="7"/>
+      <c r="AE5" s="7"/>
+      <c r="AF5" s="7"/>
+      <c r="AG5" s="7"/>
+      <c r="AH5" s="7"/>
+      <c r="AI5" s="7"/>
+      <c r="AJ5" s="7"/>
+      <c r="AK5" s="7"/>
+      <c r="AL5" s="7"/>
+      <c r="AM5" s="7"/>
+      <c r="AN5" s="7"/>
+      <c r="AO5" s="7"/>
+      <c r="AP5" s="7"/>
+      <c r="AQ5" s="7"/>
+      <c r="AR5" s="7"/>
+      <c r="AS5" s="7"/>
+      <c r="AT5" s="7"/>
+      <c r="AU5" s="7"/>
+      <c r="AV5" s="7"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="6" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="1">
         <v>7.83</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>0.78100000000000003</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="1">
         <v>18.1906573218874</v>
       </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
         <v>0.74318344737699604</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="1">
         <v>-10.74200319593316</v>
       </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
+      <c r="K6" s="1">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1">
+        <v>0</v>
+      </c>
+      <c r="M6" s="1">
         <v>2.9274438905658182</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="1">
         <v>0.51108707409410503</v>
       </c>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="7"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="7"/>
+      <c r="T6" s="7"/>
+      <c r="U6" s="7"/>
+      <c r="V6" s="7"/>
+      <c r="W6" s="7"/>
+      <c r="X6" s="7"/>
+      <c r="Y6" s="7"/>
+      <c r="Z6" s="7"/>
+      <c r="AA6" s="7"/>
+      <c r="AB6" s="7"/>
+      <c r="AC6" s="7"/>
+      <c r="AD6" s="7"/>
+      <c r="AE6" s="7"/>
+      <c r="AF6" s="7"/>
+      <c r="AG6" s="7"/>
+      <c r="AH6" s="7"/>
+      <c r="AI6" s="7"/>
+      <c r="AJ6" s="7"/>
+      <c r="AK6" s="7"/>
+      <c r="AL6" s="7"/>
+      <c r="AM6" s="7"/>
+      <c r="AN6" s="7"/>
+      <c r="AO6" s="7"/>
+      <c r="AP6" s="7"/>
+      <c r="AQ6" s="7"/>
+      <c r="AR6" s="7"/>
+      <c r="AS6" s="7"/>
+      <c r="AT6" s="7"/>
+      <c r="AU6" s="7"/>
+      <c r="AV6" s="7"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7">
+    <row r="7" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="1">
         <v>24.42</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>1.61</v>
       </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
         <v>0.78228413163897004</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="1">
         <v>-1.2400966196699801</v>
       </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
+      <c r="K7" s="1">
+        <v>0</v>
+      </c>
+      <c r="L7" s="1">
+        <v>0</v>
+      </c>
+      <c r="M7" s="1">
         <v>2.665578572672828E-3</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="1">
         <v>6.756336041409737E-2</v>
       </c>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="7"/>
+      <c r="X7" s="7"/>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="7"/>
+      <c r="AA7" s="7"/>
+      <c r="AB7" s="7"/>
+      <c r="AC7" s="7"/>
+      <c r="AD7" s="7"/>
+      <c r="AE7" s="7"/>
+      <c r="AF7" s="7"/>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="7"/>
+      <c r="AI7" s="7"/>
+      <c r="AJ7" s="7"/>
+      <c r="AK7" s="7"/>
+      <c r="AL7" s="7"/>
+      <c r="AM7" s="7"/>
+      <c r="AN7" s="7"/>
+      <c r="AO7" s="7"/>
+      <c r="AP7" s="7"/>
+      <c r="AQ7" s="7"/>
+      <c r="AR7" s="7"/>
+      <c r="AS7" s="7"/>
+      <c r="AT7" s="7"/>
+      <c r="AU7" s="7"/>
+      <c r="AV7" s="7"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8">
+    <row r="8" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="1">
         <v>25.67</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>1.65</v>
       </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
+      <c r="F8" s="1">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
         <v>0.51248941023134598</v>
       </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
+      <c r="J8" s="1">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0</v>
+      </c>
+      <c r="L8" s="1">
+        <v>0</v>
+      </c>
+      <c r="M8" s="1">
         <v>-0.17903540723894801</v>
       </c>
-      <c r="N8">
+      <c r="N8" s="1">
         <v>4.3266630611140951E-2</v>
       </c>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="7"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="7"/>
+      <c r="X8" s="7"/>
+      <c r="Y8" s="7"/>
+      <c r="Z8" s="7"/>
+      <c r="AA8" s="7"/>
+      <c r="AB8" s="7"/>
+      <c r="AC8" s="7"/>
+      <c r="AD8" s="7"/>
+      <c r="AE8" s="7"/>
+      <c r="AF8" s="7"/>
+      <c r="AG8" s="7"/>
+      <c r="AH8" s="7"/>
+      <c r="AI8" s="7"/>
+      <c r="AJ8" s="7"/>
+      <c r="AK8" s="7"/>
+      <c r="AL8" s="7"/>
+      <c r="AM8" s="7"/>
+      <c r="AN8" s="7"/>
+      <c r="AO8" s="7"/>
+      <c r="AP8" s="7"/>
+      <c r="AQ8" s="7"/>
+      <c r="AR8" s="7"/>
+      <c r="AS8" s="7"/>
+      <c r="AT8" s="7"/>
+      <c r="AU8" s="7"/>
+      <c r="AV8" s="7"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9">
+    <row r="9" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="3">
         <v>5.33</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="3">
         <v>0.11600000000000001</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="3">
         <v>25.495764015931599</v>
       </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
         <v>0.117572499185402</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="3">
         <v>-21.693553638419498</v>
       </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
+      <c r="K9" s="3">
+        <v>0</v>
+      </c>
+      <c r="L9" s="3">
+        <v>0</v>
+      </c>
+      <c r="M9" s="3">
         <v>0.43860413898537359</v>
       </c>
-      <c r="N9">
+      <c r="N9" s="3">
         <v>2.4352700156364631E-2</v>
       </c>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
+      <c r="R9" s="7"/>
+      <c r="S9" s="7"/>
+      <c r="T9" s="7"/>
+      <c r="U9" s="7"/>
+      <c r="V9" s="7"/>
+      <c r="W9" s="7"/>
+      <c r="X9" s="7"/>
+      <c r="Y9" s="7"/>
+      <c r="Z9" s="7"/>
+      <c r="AA9" s="7"/>
+      <c r="AB9" s="7"/>
+      <c r="AC9" s="7"/>
+      <c r="AD9" s="7"/>
+      <c r="AE9" s="7"/>
+      <c r="AF9" s="7"/>
+      <c r="AG9" s="7"/>
+      <c r="AH9" s="7"/>
+      <c r="AI9" s="7"/>
+      <c r="AJ9" s="7"/>
+      <c r="AK9" s="7"/>
+      <c r="AL9" s="7"/>
+      <c r="AM9" s="7"/>
+      <c r="AN9" s="7"/>
+      <c r="AO9" s="7"/>
+      <c r="AP9" s="7"/>
+      <c r="AQ9" s="7"/>
+      <c r="AR9" s="7"/>
+      <c r="AS9" s="7"/>
+      <c r="AT9" s="7"/>
+      <c r="AU9" s="7"/>
+      <c r="AV9" s="7"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10">
+    <row r="10" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="3">
         <v>6.58</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="3">
         <v>0.28399999999999997</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="3">
         <v>23.297399473737801</v>
       </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
+      <c r="G10" s="3">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3">
         <v>0.25116650374714899</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="3">
         <v>-11.889478324466181</v>
       </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
+      <c r="K10" s="3">
+        <v>0</v>
+      </c>
+      <c r="L10" s="3">
+        <v>0</v>
+      </c>
+      <c r="M10" s="3">
         <v>0.72252030590452676</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="3">
         <v>0.18171984856679291</v>
       </c>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="7"/>
+      <c r="T10" s="7"/>
+      <c r="U10" s="7"/>
+      <c r="V10" s="7"/>
+      <c r="W10" s="7"/>
+      <c r="X10" s="7"/>
+      <c r="Y10" s="7"/>
+      <c r="Z10" s="7"/>
+      <c r="AA10" s="7"/>
+      <c r="AB10" s="7"/>
+      <c r="AC10" s="7"/>
+      <c r="AD10" s="7"/>
+      <c r="AE10" s="7"/>
+      <c r="AF10" s="7"/>
+      <c r="AG10" s="7"/>
+      <c r="AH10" s="7"/>
+      <c r="AI10" s="7"/>
+      <c r="AJ10" s="7"/>
+      <c r="AK10" s="7"/>
+      <c r="AL10" s="7"/>
+      <c r="AM10" s="7"/>
+      <c r="AN10" s="7"/>
+      <c r="AO10" s="7"/>
+      <c r="AP10" s="7"/>
+      <c r="AQ10" s="7"/>
+      <c r="AR10" s="7"/>
+      <c r="AS10" s="7"/>
+      <c r="AT10" s="7"/>
+      <c r="AU10" s="7"/>
+      <c r="AV10" s="7"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11">
+    <row r="11" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="3">
         <v>7.33</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="3">
         <v>0.48199999999999998</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="3">
         <v>21.805346498762599</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
         <v>0.150483507749371</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="3">
         <v>0.22735156771180801</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="3">
         <v>0.41082763115021198</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="3">
         <v>-7.0230749478357613</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="3">
         <v>0.70832401467154416</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="3">
         <v>1.0701410247008969</v>
       </c>
-      <c r="M11">
+      <c r="M11" s="3">
         <v>0.75152295717000372</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="3">
         <v>0.35694970254191449</v>
       </c>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="7"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="7"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="7"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="7"/>
+      <c r="X11" s="7"/>
+      <c r="Y11" s="7"/>
+      <c r="Z11" s="7"/>
+      <c r="AA11" s="7"/>
+      <c r="AB11" s="7"/>
+      <c r="AC11" s="7"/>
+      <c r="AD11" s="7"/>
+      <c r="AE11" s="7"/>
+      <c r="AF11" s="7"/>
+      <c r="AG11" s="7"/>
+      <c r="AH11" s="7"/>
+      <c r="AI11" s="7"/>
+      <c r="AJ11" s="7"/>
+      <c r="AK11" s="7"/>
+      <c r="AL11" s="7"/>
+      <c r="AM11" s="7"/>
+      <c r="AN11" s="7"/>
+      <c r="AO11" s="7"/>
+      <c r="AP11" s="7"/>
+      <c r="AQ11" s="7"/>
+      <c r="AR11" s="7"/>
+      <c r="AS11" s="7"/>
+      <c r="AT11" s="7"/>
+      <c r="AU11" s="7"/>
+      <c r="AV11" s="7"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12">
+    <row r="12" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="3">
         <v>8.08</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="3">
         <v>0.76</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="3">
         <v>18.4534094054106</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>0.268379917869917</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="3">
         <v>0.26737825216811201</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="3">
         <v>0.72037471489084404</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="3">
         <v>-9.7307450382342413</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="3">
         <v>0.34225579891742258</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="3">
         <v>0.11619832064946389</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="3">
         <v>0.89862180146013859</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="3">
         <v>0.50117180457905175</v>
       </c>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7"/>
+      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="7"/>
+      <c r="V12" s="7"/>
+      <c r="W12" s="7"/>
+      <c r="X12" s="7"/>
+      <c r="Y12" s="7"/>
+      <c r="Z12" s="7"/>
+      <c r="AA12" s="7"/>
+      <c r="AB12" s="7"/>
+      <c r="AC12" s="7"/>
+      <c r="AD12" s="7"/>
+      <c r="AE12" s="7"/>
+      <c r="AF12" s="7"/>
+      <c r="AG12" s="7"/>
+      <c r="AH12" s="7"/>
+      <c r="AI12" s="7"/>
+      <c r="AJ12" s="7"/>
+      <c r="AK12" s="7"/>
+      <c r="AL12" s="7"/>
+      <c r="AM12" s="7"/>
+      <c r="AN12" s="7"/>
+      <c r="AO12" s="7"/>
+      <c r="AP12" s="7"/>
+      <c r="AQ12" s="7"/>
+      <c r="AR12" s="7"/>
+      <c r="AS12" s="7"/>
+      <c r="AT12" s="7"/>
+      <c r="AU12" s="7"/>
+      <c r="AV12" s="7"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13">
+    <row r="13" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="3">
         <v>24.42</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="3">
         <v>1.6</v>
       </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
         <v>0.37832825539806603</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="3">
         <v>0.173982655103402</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="3">
         <v>0.808351254480287</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="3">
         <v>-1.2940339039129729</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="3">
         <v>7.7100590635883204E-3</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="3">
         <v>-6.5493083918949967E-3</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="3">
         <v>6.1693003431821918E-3</v>
       </c>
-      <c r="N13">
+      <c r="N13" s="3">
         <v>6.9507286018510112E-2</v>
       </c>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="7"/>
+      <c r="R13" s="7"/>
+      <c r="S13" s="7"/>
+      <c r="T13" s="7"/>
+      <c r="U13" s="7"/>
+      <c r="V13" s="7"/>
+      <c r="W13" s="7"/>
+      <c r="X13" s="7"/>
+      <c r="Y13" s="7"/>
+      <c r="Z13" s="7"/>
+      <c r="AA13" s="7"/>
+      <c r="AB13" s="7"/>
+      <c r="AC13" s="7"/>
+      <c r="AD13" s="7"/>
+      <c r="AE13" s="7"/>
+      <c r="AF13" s="7"/>
+      <c r="AG13" s="7"/>
+      <c r="AH13" s="7"/>
+      <c r="AI13" s="7"/>
+      <c r="AJ13" s="7"/>
+      <c r="AK13" s="7"/>
+      <c r="AL13" s="7"/>
+      <c r="AM13" s="7"/>
+      <c r="AN13" s="7"/>
+      <c r="AO13" s="7"/>
+      <c r="AP13" s="7"/>
+      <c r="AQ13" s="7"/>
+      <c r="AR13" s="7"/>
+      <c r="AS13" s="7"/>
+      <c r="AT13" s="7"/>
+      <c r="AU13" s="7"/>
+      <c r="AV13" s="7"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14">
+    <row r="14" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="3">
         <v>25.67</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="3">
         <v>1.6379999999999999</v>
       </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14">
+      <c r="F14" s="3">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3">
         <v>0.36110743144787399</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="3">
         <v>0.18398932621747799</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="3">
         <v>0.52878136200716797</v>
       </c>
-      <c r="J14">
-        <v>0</v>
-      </c>
-      <c r="K14">
+      <c r="J14" s="3">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3">
         <v>-1.150535868858016E-2</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="3">
         <v>6.6855303079046066E-3</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="3">
         <v>-0.18678269406471421</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="3">
         <v>4.1103299080583897E-2</v>
       </c>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="7"/>
+      <c r="R14" s="7"/>
+      <c r="S14" s="7"/>
+      <c r="T14" s="7"/>
+      <c r="U14" s="7"/>
+      <c r="V14" s="7"/>
+      <c r="W14" s="7"/>
+      <c r="X14" s="7"/>
+      <c r="Y14" s="7"/>
+      <c r="Z14" s="7"/>
+      <c r="AA14" s="7"/>
+      <c r="AB14" s="7"/>
+      <c r="AC14" s="7"/>
+      <c r="AD14" s="7"/>
+      <c r="AE14" s="7"/>
+      <c r="AF14" s="7"/>
+      <c r="AG14" s="7"/>
+      <c r="AH14" s="7"/>
+      <c r="AI14" s="7"/>
+      <c r="AJ14" s="7"/>
+      <c r="AK14" s="7"/>
+      <c r="AL14" s="7"/>
+      <c r="AM14" s="7"/>
+      <c r="AN14" s="7"/>
+      <c r="AO14" s="7"/>
+      <c r="AP14" s="7"/>
+      <c r="AQ14" s="7"/>
+      <c r="AR14" s="7"/>
+      <c r="AS14" s="7"/>
+      <c r="AT14" s="7"/>
+      <c r="AU14" s="7"/>
+      <c r="AV14" s="7"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15">
+    <row r="15" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="2">
         <v>8.08</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="2">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="2">
         <v>25.080521009105698</v>
       </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
+      <c r="G15" s="2">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2">
         <v>-43.440873874032498</v>
       </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-      <c r="N15">
+      <c r="K15" s="2">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2">
+        <v>0</v>
+      </c>
+      <c r="N15" s="2">
         <v>1.3386952540575851E-3</v>
       </c>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+      <c r="Q15" s="7"/>
+      <c r="R15" s="7"/>
+      <c r="S15" s="7"/>
+      <c r="T15" s="7"/>
+      <c r="U15" s="7"/>
+      <c r="V15" s="7"/>
+      <c r="W15" s="7"/>
+      <c r="X15" s="7"/>
+      <c r="Y15" s="7"/>
+      <c r="Z15" s="7"/>
+      <c r="AA15" s="7"/>
+      <c r="AB15" s="7"/>
+      <c r="AC15" s="7"/>
+      <c r="AD15" s="7"/>
+      <c r="AE15" s="7"/>
+      <c r="AF15" s="7"/>
+      <c r="AG15" s="7"/>
+      <c r="AH15" s="7"/>
+      <c r="AI15" s="7"/>
+      <c r="AJ15" s="7"/>
+      <c r="AK15" s="7"/>
+      <c r="AL15" s="7"/>
+      <c r="AM15" s="7"/>
+      <c r="AN15" s="7"/>
+      <c r="AO15" s="7"/>
+      <c r="AP15" s="7"/>
+      <c r="AQ15" s="7"/>
+      <c r="AR15" s="7"/>
+      <c r="AS15" s="7"/>
+      <c r="AT15" s="7"/>
+      <c r="AU15" s="7"/>
+      <c r="AV15" s="7"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16">
+    <row r="16" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="2">
         <v>16</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="2">
         <v>0.26</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="2">
         <v>24.474454777917</v>
       </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-      <c r="J16">
+      <c r="G16" s="2">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2">
         <v>-0.71851445637823264</v>
       </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16">
-        <v>0</v>
-      </c>
-      <c r="N16">
+      <c r="K16" s="2">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2">
+        <v>0</v>
+      </c>
+      <c r="N16" s="2">
         <v>3.9606448476107753E-2</v>
       </c>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="7"/>
+      <c r="R16" s="7"/>
+      <c r="S16" s="7"/>
+      <c r="T16" s="7"/>
+      <c r="U16" s="7"/>
+      <c r="V16" s="7"/>
+      <c r="W16" s="7"/>
+      <c r="X16" s="7"/>
+      <c r="Y16" s="7"/>
+      <c r="Z16" s="7"/>
+      <c r="AA16" s="7"/>
+      <c r="AB16" s="7"/>
+      <c r="AC16" s="7"/>
+      <c r="AD16" s="7"/>
+      <c r="AE16" s="7"/>
+      <c r="AF16" s="7"/>
+      <c r="AG16" s="7"/>
+      <c r="AH16" s="7"/>
+      <c r="AI16" s="7"/>
+      <c r="AJ16" s="7"/>
+      <c r="AK16" s="7"/>
+      <c r="AL16" s="7"/>
+      <c r="AM16" s="7"/>
+      <c r="AN16" s="7"/>
+      <c r="AO16" s="7"/>
+      <c r="AP16" s="7"/>
+      <c r="AQ16" s="7"/>
+      <c r="AR16" s="7"/>
+      <c r="AS16" s="7"/>
+      <c r="AT16" s="7"/>
+      <c r="AU16" s="7"/>
+      <c r="AV16" s="7"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17">
+    <row r="17" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="2">
         <v>18.25</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="2">
         <v>0.38300000000000001</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="2">
         <v>23.767032760625099</v>
       </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="I17">
-        <v>0</v>
-      </c>
-      <c r="J17">
+      <c r="G17" s="2">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
         <v>-1.3222640015706311</v>
       </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17">
+      <c r="K17" s="2">
+        <v>0</v>
+      </c>
+      <c r="L17" s="2">
+        <v>0</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0</v>
+      </c>
+      <c r="N17" s="2">
         <v>7.3913827294032813E-2</v>
       </c>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
+      <c r="V17" s="7"/>
+      <c r="W17" s="7"/>
+      <c r="X17" s="7"/>
+      <c r="Y17" s="7"/>
+      <c r="Z17" s="7"/>
+      <c r="AA17" s="7"/>
+      <c r="AB17" s="7"/>
+      <c r="AC17" s="7"/>
+      <c r="AD17" s="7"/>
+      <c r="AE17" s="7"/>
+      <c r="AF17" s="7"/>
+      <c r="AG17" s="7"/>
+      <c r="AH17" s="7"/>
+      <c r="AI17" s="7"/>
+      <c r="AJ17" s="7"/>
+      <c r="AK17" s="7"/>
+      <c r="AL17" s="7"/>
+      <c r="AM17" s="7"/>
+      <c r="AN17" s="7"/>
+      <c r="AO17" s="7"/>
+      <c r="AP17" s="7"/>
+      <c r="AQ17" s="7"/>
+      <c r="AR17" s="7"/>
+      <c r="AS17" s="7"/>
+      <c r="AT17" s="7"/>
+      <c r="AU17" s="7"/>
+      <c r="AV17" s="7"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18">
+    <row r="18" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>22.33</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="2">
         <v>0.65700000000000003</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="2">
         <v>21.462739990849801</v>
       </c>
-      <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="H18">
-        <v>0</v>
-      </c>
-      <c r="I18">
-        <v>0</v>
-      </c>
-      <c r="J18">
+      <c r="G18" s="2">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2">
         <v>-1.4685111485699349</v>
       </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="N18">
+      <c r="K18" s="2">
+        <v>0</v>
+      </c>
+      <c r="L18" s="2">
+        <v>0</v>
+      </c>
+      <c r="M18" s="2">
+        <v>0</v>
+      </c>
+      <c r="N18" s="2">
         <v>9.0801599168602046E-2</v>
       </c>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="7"/>
+      <c r="T18" s="7"/>
+      <c r="U18" s="7"/>
+      <c r="V18" s="7"/>
+      <c r="W18" s="7"/>
+      <c r="X18" s="7"/>
+      <c r="Y18" s="7"/>
+      <c r="Z18" s="7"/>
+      <c r="AA18" s="7"/>
+      <c r="AB18" s="7"/>
+      <c r="AC18" s="7"/>
+      <c r="AD18" s="7"/>
+      <c r="AE18" s="7"/>
+      <c r="AF18" s="7"/>
+      <c r="AG18" s="7"/>
+      <c r="AH18" s="7"/>
+      <c r="AI18" s="7"/>
+      <c r="AJ18" s="7"/>
+      <c r="AK18" s="7"/>
+      <c r="AL18" s="7"/>
+      <c r="AM18" s="7"/>
+      <c r="AN18" s="7"/>
+      <c r="AO18" s="7"/>
+      <c r="AP18" s="7"/>
+      <c r="AQ18" s="7"/>
+      <c r="AR18" s="7"/>
+      <c r="AS18" s="7"/>
+      <c r="AT18" s="7"/>
+      <c r="AU18" s="7"/>
+      <c r="AV18" s="7"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19">
+    <row r="19" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="2">
         <v>24.42</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="2">
         <v>1.02</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="2">
         <v>16.5739291092694</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="2">
         <v>0.29752285070870299</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="2">
         <v>0.23002001334222799</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="2">
         <v>0.28766047572499198</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="2">
         <v>-3.771872308096492</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="2">
         <v>0.22954829483019509</v>
       </c>
-      <c r="L19">
+      <c r="L19" s="2">
         <v>0.1774677195844126</v>
       </c>
-      <c r="M19">
+      <c r="M19" s="2">
         <v>0.22193916042221859</v>
       </c>
-      <c r="N19">
+      <c r="N19" s="2">
         <v>0.2348353306196802</v>
       </c>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="7"/>
+      <c r="R19" s="7"/>
+      <c r="S19" s="7"/>
+      <c r="T19" s="7"/>
+      <c r="U19" s="7"/>
+      <c r="V19" s="7"/>
+      <c r="W19" s="7"/>
+      <c r="X19" s="7"/>
+      <c r="Y19" s="7"/>
+      <c r="Z19" s="7"/>
+      <c r="AA19" s="7"/>
+      <c r="AB19" s="7"/>
+      <c r="AC19" s="7"/>
+      <c r="AD19" s="7"/>
+      <c r="AE19" s="7"/>
+      <c r="AF19" s="7"/>
+      <c r="AG19" s="7"/>
+      <c r="AH19" s="7"/>
+      <c r="AI19" s="7"/>
+      <c r="AJ19" s="7"/>
+      <c r="AK19" s="7"/>
+      <c r="AL19" s="7"/>
+      <c r="AM19" s="7"/>
+      <c r="AN19" s="7"/>
+      <c r="AO19" s="7"/>
+      <c r="AP19" s="7"/>
+      <c r="AQ19" s="7"/>
+      <c r="AR19" s="7"/>
+      <c r="AS19" s="7"/>
+      <c r="AT19" s="7"/>
+      <c r="AU19" s="7"/>
+      <c r="AV19" s="7"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20">
+    <row r="20" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="2">
         <v>28.33</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="2">
         <v>1.4139999999999999</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="2">
         <v>9.7241287188137502</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="2">
         <v>0.39819843687905698</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="2">
         <v>0.40747164776517703</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="2">
         <v>1.1374486803519099</v>
       </c>
-      <c r="J20">
+      <c r="J20" s="2">
         <v>-1.946317456384979</v>
       </c>
-      <c r="K20">
+      <c r="K20" s="2">
         <v>2.8606184067520791E-2</v>
       </c>
-      <c r="L20">
+      <c r="L20" s="2">
         <v>5.0421500489659779E-2</v>
       </c>
-      <c r="M20">
+      <c r="M20" s="2">
         <v>0.24146070288413171</v>
       </c>
-      <c r="N20">
+      <c r="N20" s="2">
         <v>0.13624562388738509</v>
       </c>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7"/>
+      <c r="R20" s="7"/>
+      <c r="S20" s="7"/>
+      <c r="T20" s="7"/>
+      <c r="U20" s="7"/>
+      <c r="V20" s="7"/>
+      <c r="W20" s="7"/>
+      <c r="X20" s="7"/>
+      <c r="Y20" s="7"/>
+      <c r="Z20" s="7"/>
+      <c r="AA20" s="7"/>
+      <c r="AB20" s="7"/>
+      <c r="AC20" s="7"/>
+      <c r="AD20" s="7"/>
+      <c r="AE20" s="7"/>
+      <c r="AF20" s="7"/>
+      <c r="AG20" s="7"/>
+      <c r="AH20" s="7"/>
+      <c r="AI20" s="7"/>
+      <c r="AJ20" s="7"/>
+      <c r="AK20" s="7"/>
+      <c r="AL20" s="7"/>
+      <c r="AM20" s="7"/>
+      <c r="AN20" s="7"/>
+      <c r="AO20" s="7"/>
+      <c r="AP20" s="7"/>
+      <c r="AQ20" s="7"/>
+      <c r="AR20" s="7"/>
+      <c r="AS20" s="7"/>
+      <c r="AT20" s="7"/>
+      <c r="AU20" s="7"/>
+      <c r="AV20" s="7"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21">
+    <row r="21" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="2">
         <v>31.67</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="2">
         <v>1.522</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="2">
         <v>4.5216048047574997</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="2">
         <v>0.346535965028481</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="2">
         <v>0.29339559706471002</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="2">
         <v>1.79987943955686</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="2">
         <v>-1.434645697759156</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="2">
         <v>-1.424642042985734E-2</v>
       </c>
-      <c r="L21">
+      <c r="L21" s="2">
         <v>-3.1457561379507538E-2</v>
       </c>
-      <c r="M21">
+      <c r="M21" s="2">
         <v>0.18267161371215129</v>
       </c>
-      <c r="N21">
+      <c r="N21" s="2">
         <v>4.3720023446886642E-2</v>
       </c>
+      <c r="O21" s="7"/>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="7"/>
+      <c r="R21" s="7"/>
+      <c r="S21" s="7"/>
+      <c r="T21" s="7"/>
+      <c r="U21" s="7"/>
+      <c r="V21" s="7"/>
+      <c r="W21" s="7"/>
+      <c r="X21" s="7"/>
+      <c r="Y21" s="7"/>
+      <c r="Z21" s="7"/>
+      <c r="AA21" s="7"/>
+      <c r="AB21" s="7"/>
+      <c r="AC21" s="7"/>
+      <c r="AD21" s="7"/>
+      <c r="AE21" s="7"/>
+      <c r="AF21" s="7"/>
+      <c r="AG21" s="7"/>
+      <c r="AH21" s="7"/>
+      <c r="AI21" s="7"/>
+      <c r="AJ21" s="7"/>
+      <c r="AK21" s="7"/>
+      <c r="AL21" s="7"/>
+      <c r="AM21" s="7"/>
+      <c r="AN21" s="7"/>
+      <c r="AO21" s="7"/>
+      <c r="AP21" s="7"/>
+      <c r="AQ21" s="7"/>
+      <c r="AR21" s="7"/>
+      <c r="AS21" s="7"/>
+      <c r="AT21" s="7"/>
+      <c r="AU21" s="7"/>
+      <c r="AV21" s="7"/>
+    </row>
+    <row r="22" spans="1:48" x14ac:dyDescent="0.3">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Excel con inoculos, imagenes escher
</commit_message>
<xml_diff>
--- a/Data/HPLC_results/Resultados_Procesados.xlsx
+++ b/Data/HPLC_results/Resultados_Procesados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\yannis\CNB\CNB\Data\HPLC_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7351E0C0-A6A4-4543-88A6-7B5A1A59EA73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62692C68-B477-49AB-96BB-EC698085453F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="1944" windowWidth="17352" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="41">
   <si>
     <t>#</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>0.815022</t>
+  </si>
+  <si>
+    <t>Inóculo</t>
   </si>
 </sst>
 </file>
@@ -173,7 +176,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -210,8 +213,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -234,11 +243,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -248,6 +266,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="11" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -554,6 +577,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="14" max="14" width="8.88671875" customWidth="1"/>
+    <col min="16" max="16" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:48" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -600,7 +624,9 @@
         <v>13</v>
       </c>
       <c r="O1"/>
-      <c r="P1"/>
+      <c r="P1" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="Q1"/>
       <c r="R1"/>
       <c r="S1"/>
@@ -676,7 +702,7 @@
       </c>
       <c r="N2" s="6"/>
       <c r="O2"/>
-      <c r="P2"/>
+      <c r="P2" s="8"/>
       <c r="Q2"/>
       <c r="R2"/>
       <c r="S2"/>
@@ -754,7 +780,10 @@
         <v>3.323128875503923E-2</v>
       </c>
       <c r="O3"/>
-      <c r="P3"/>
+      <c r="P3" s="9">
+        <f>E3*8*100000000</f>
+        <v>120800000</v>
+      </c>
       <c r="Q3"/>
       <c r="R3"/>
       <c r="S3"/>
@@ -832,7 +861,7 @@
         <v>0.2314764737696052</v>
       </c>
       <c r="O4"/>
-      <c r="P4"/>
+      <c r="P4" s="8"/>
       <c r="Q4"/>
       <c r="R4"/>
       <c r="S4"/>
@@ -911,7 +940,10 @@
         <v>0.40923021453037672</v>
       </c>
       <c r="O5"/>
-      <c r="P5"/>
+      <c r="P5" s="9">
+        <f t="shared" ref="P4:P21" si="0">E5*8*100000000</f>
+        <v>473600000</v>
+      </c>
       <c r="Q5"/>
       <c r="R5"/>
       <c r="S5"/>
@@ -989,7 +1021,7 @@
         <v>0.51108707409410503</v>
       </c>
       <c r="O6"/>
-      <c r="P6"/>
+      <c r="P6" s="8"/>
       <c r="Q6"/>
       <c r="R6"/>
       <c r="S6"/>
@@ -1067,7 +1099,7 @@
         <v>6.756336041409737E-2</v>
       </c>
       <c r="O7"/>
-      <c r="P7"/>
+      <c r="P7" s="8"/>
       <c r="Q7"/>
       <c r="R7"/>
       <c r="S7"/>
@@ -1145,7 +1177,7 @@
         <v>4.3266630611140951E-2</v>
       </c>
       <c r="O8"/>
-      <c r="P8"/>
+      <c r="P8" s="8"/>
       <c r="Q8"/>
       <c r="R8"/>
       <c r="S8"/>
@@ -1223,7 +1255,10 @@
         <v>2.4352700156364631E-2</v>
       </c>
       <c r="O9"/>
-      <c r="P9"/>
+      <c r="P9" s="9">
+        <f t="shared" si="0"/>
+        <v>92800000</v>
+      </c>
       <c r="Q9"/>
       <c r="R9"/>
       <c r="S9"/>
@@ -1301,7 +1336,7 @@
         <v>0.18171984856679291</v>
       </c>
       <c r="O10"/>
-      <c r="P10"/>
+      <c r="P10" s="8"/>
       <c r="Q10"/>
       <c r="R10"/>
       <c r="S10"/>
@@ -1379,7 +1414,10 @@
         <v>0.35694970254191449</v>
       </c>
       <c r="O11"/>
-      <c r="P11"/>
+      <c r="P11" s="9">
+        <f t="shared" si="0"/>
+        <v>385600000</v>
+      </c>
       <c r="Q11"/>
       <c r="R11"/>
       <c r="S11"/>
@@ -1457,7 +1495,7 @@
         <v>0.50117180457905175</v>
       </c>
       <c r="O12"/>
-      <c r="P12"/>
+      <c r="P12" s="8"/>
       <c r="Q12"/>
       <c r="R12"/>
       <c r="S12"/>
@@ -1535,7 +1573,7 @@
         <v>6.9507286018510112E-2</v>
       </c>
       <c r="O13"/>
-      <c r="P13"/>
+      <c r="P13" s="8"/>
       <c r="Q13"/>
       <c r="R13"/>
       <c r="S13"/>
@@ -1613,7 +1651,7 @@
         <v>4.1103299080583897E-2</v>
       </c>
       <c r="O14"/>
-      <c r="P14"/>
+      <c r="P14" s="8"/>
       <c r="Q14"/>
       <c r="R14"/>
       <c r="S14"/>
@@ -1691,7 +1729,10 @@
         <v>1.3386952540575851E-3</v>
       </c>
       <c r="O15"/>
-      <c r="P15"/>
+      <c r="P15" s="9">
+        <f t="shared" si="0"/>
+        <v>22400000</v>
+      </c>
       <c r="Q15"/>
       <c r="R15"/>
       <c r="S15"/>
@@ -1769,7 +1810,7 @@
         <v>3.9606448476107753E-2</v>
       </c>
       <c r="O16"/>
-      <c r="P16"/>
+      <c r="P16" s="8"/>
       <c r="Q16"/>
       <c r="R16"/>
       <c r="S16"/>
@@ -1847,7 +1888,10 @@
         <v>7.3913827294032813E-2</v>
       </c>
       <c r="O17"/>
-      <c r="P17"/>
+      <c r="P17" s="9">
+        <f t="shared" si="0"/>
+        <v>306400000</v>
+      </c>
       <c r="Q17"/>
       <c r="R17"/>
       <c r="S17"/>
@@ -1925,7 +1969,7 @@
         <v>9.0801599168602046E-2</v>
       </c>
       <c r="O18"/>
-      <c r="P18"/>
+      <c r="P18" s="8"/>
       <c r="Q18"/>
       <c r="R18"/>
       <c r="S18"/>
@@ -2003,7 +2047,7 @@
         <v>0.2348353306196802</v>
       </c>
       <c r="O19"/>
-      <c r="P19"/>
+      <c r="P19" s="8"/>
       <c r="Q19"/>
       <c r="R19"/>
       <c r="S19"/>
@@ -2081,7 +2125,7 @@
         <v>0.13624562388738509</v>
       </c>
       <c r="O20"/>
-      <c r="P20"/>
+      <c r="P20" s="8"/>
       <c r="Q20"/>
       <c r="R20"/>
       <c r="S20"/>
@@ -2159,7 +2203,7 @@
         <v>4.3720023446886642E-2</v>
       </c>
       <c r="O21"/>
-      <c r="P21"/>
+      <c r="P21" s="8"/>
       <c r="Q21"/>
       <c r="R21"/>
       <c r="S21"/>

</xml_diff>